<commit_message>
New prospective LCIs added with premise 2.5.1
</commit_message>
<xml_diff>
--- a/data/LCIs/Lai_2025/Co_LCIs_BW_Final_v1.xlsx
+++ b/data/LCIs/Lai_2025/Co_LCIs_BW_Final_v1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://brgm365.sharepoint.com/sites/RPPEXIMPMET/Documents partages/General/P2/05_Produits/Article_LCI data/Final LCI datasets/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://polymtlca-my.sharepoint.com/personal/marin_pellan_polymtl_ca/Documents/POST_DOC/CODE/fasc_metal_sustainability/data/LCIs/Lai_2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="156" documentId="8_{0C7C91A2-ADF9-4192-ADD6-8FFEE2FDF270}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{86389B91-EA31-44A8-A791-CB1777367D29}"/>
+  <xr:revisionPtr revIDLastSave="188" documentId="8_{0C7C91A2-ADF9-4192-ADD6-8FFEE2FDF270}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3ECC0D64-B90C-4E32-BCD0-5E0A7C6B6311}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="836" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="836" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Note" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1887" uniqueCount="256">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1899" uniqueCount="254">
   <si>
     <t>Activity</t>
   </si>
@@ -332,9 +332,6 @@
   </si>
   <si>
     <t>Oxidized scrap</t>
-  </si>
-  <si>
-    <t>Europe</t>
   </si>
   <si>
     <t>RER</t>
@@ -932,9 +929,6 @@
     <t>Cu/Co ore mining in DRC and CoSO4 production in China/Tongxiang</t>
   </si>
   <si>
-    <t>CD-CN</t>
-  </si>
-  <si>
     <t>[C+P] Cobalt hydroxide (Co(OH)2) production - Hydrometallurgy</t>
   </si>
   <si>
@@ -1061,9 +1055,6 @@
   </si>
   <si>
     <t>Cu/Co ore mining in DRC and Co production</t>
-  </si>
-  <si>
-    <t>CD-CN-GLO</t>
   </si>
   <si>
     <t>This unit process is allocated, but with unknown allocation factors (not provided in the original data source).</t>
@@ -2270,6 +2261,9 @@
   </si>
   <si>
     <t>PR7_Co(OH)2_Europe_Recycling</t>
+  </si>
+  <si>
+    <t>Europe witout Switzerland</t>
   </si>
 </sst>
 </file>
@@ -2631,6 +2625,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
   <a:themeElements>
@@ -2907,12 +2905,12 @@
   <sheetData>
     <row r="1" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="28" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="C2" s="29"/>
       <c r="D2" s="29"/>
@@ -3455,10 +3453,10 @@
     <row r="32" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="33" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B33" s="16" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="C33" s="17" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="D33" s="18"/>
       <c r="E33" s="18"/>
@@ -3471,10 +3469,10 @@
     </row>
     <row r="34" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B34" s="20" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="D34" s="21"/>
       <c r="E34" s="21"/>
@@ -3487,10 +3485,10 @@
     </row>
     <row r="35" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B35" s="20" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D35" s="21"/>
       <c r="E35" s="21"/>
@@ -3503,10 +3501,10 @@
     </row>
     <row r="36" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B36" s="26" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D36" s="21"/>
       <c r="E36" s="21"/>
@@ -3519,10 +3517,10 @@
     </row>
     <row r="37" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B37" s="26" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="D37" s="21"/>
       <c r="E37" s="21"/>
@@ -3535,10 +3533,10 @@
     </row>
     <row r="38" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B38" s="26" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="D38" s="21"/>
       <c r="E38" s="21"/>
@@ -3551,7 +3549,7 @@
     </row>
     <row r="39" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B39" s="20" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="C39" s="4" t="s">
         <v>91</v>
@@ -3567,7 +3565,7 @@
     </row>
     <row r="40" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B40" s="20" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="C40" s="4" t="s">
         <v>94</v>
@@ -3583,10 +3581,10 @@
     </row>
     <row r="41" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B41" s="27" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="C41" s="23" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D41" s="24"/>
       <c r="E41" s="24"/>
@@ -3625,7 +3623,7 @@
   <cols>
     <col min="1" max="1" width="88.28515625" style="4" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="36.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.7109375" style="4" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" style="4" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8.7109375" style="4" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9" style="4" bestFit="1" customWidth="1"/>
@@ -3654,7 +3652,7 @@
         <v>0</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
@@ -3662,7 +3660,7 @@
         <v>1</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
@@ -3811,9 +3809,8 @@
         <f>'PR2_CoSO4_CD-CN_Tongxiang'!B67</f>
         <v>CoSO4</v>
       </c>
-      <c r="C13" s="4" t="str">
-        <f>'PR2_CoSO4_CD-CN_Tongxiang'!C67</f>
-        <v>CD-CN</v>
+      <c r="C13" s="4" t="s">
+        <v>141</v>
       </c>
       <c r="D13" s="4">
         <v>0.15164499389936367</v>
@@ -3839,9 +3836,8 @@
         <f>'PR3_Co3O4_CD-CN_Quzhou'!B28</f>
         <v>Co3O4</v>
       </c>
-      <c r="C14" s="4" t="str">
-        <f>'PR3_Co3O4_CD-CN_Quzhou'!C28</f>
-        <v>CD-CN</v>
+      <c r="C14" s="4" t="s">
+        <v>141</v>
       </c>
       <c r="D14" s="4">
         <v>0.15679843399801235</v>
@@ -3867,9 +3863,8 @@
         <f>'PR4_Co_CD-CN-GLO'!B20</f>
         <v>Co metal</v>
       </c>
-      <c r="C15" s="4" t="str">
-        <f>'PR4_Co_CD-CN-GLO'!C20</f>
-        <v>CD-CN-GLO</v>
+      <c r="C15" s="4" t="s">
+        <v>141</v>
       </c>
       <c r="D15" s="4">
         <v>0.5100041641971339</v>
@@ -3953,7 +3948,7 @@
       </c>
       <c r="C18" s="4" t="str">
         <f>'PR7_Co(OH)2_Europe_Recycling'!C103</f>
-        <v>Europe</v>
+        <v>Europe witout Switzerland</v>
       </c>
       <c r="D18" s="4">
         <v>6.2643907715534755E-3</v>
@@ -3976,7 +3971,7 @@
         <v>0</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.25">
@@ -3984,7 +3979,7 @@
         <v>1</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.25">
@@ -4133,9 +4128,8 @@
         <f>'PR2_CoSO4_CD-CN_Tongxiang'!B80</f>
         <v>CoSO4 (Co content)</v>
       </c>
-      <c r="C30" s="4" t="str">
-        <f>'PR2_CoSO4_CD-CN_Tongxiang'!C80</f>
-        <v>CD-CN</v>
+      <c r="C30" s="4" t="s">
+        <v>141</v>
       </c>
       <c r="D30" s="4">
         <v>0.15164499389936367</v>
@@ -4161,9 +4155,8 @@
         <f>'PR3_Co3O4_CD-CN_Quzhou'!B42</f>
         <v>Co3O4 (Co content)</v>
       </c>
-      <c r="C31" s="4" t="str">
-        <f>'PR3_Co3O4_CD-CN_Quzhou'!C42</f>
-        <v>CD-CN</v>
+      <c r="C31" s="4" t="s">
+        <v>141</v>
       </c>
       <c r="D31" s="4">
         <v>0.15679843399801235</v>
@@ -4189,9 +4182,8 @@
         <f>'PR4_Co_CD-CN-GLO'!B20</f>
         <v>Co metal</v>
       </c>
-      <c r="C32" s="4" t="str">
-        <f>'PR4_Co_CD-CN-GLO'!C20</f>
-        <v>CD-CN-GLO</v>
+      <c r="C32" s="4" t="s">
+        <v>141</v>
       </c>
       <c r="D32" s="4">
         <v>0.5100041641971339</v>
@@ -4275,7 +4267,7 @@
       </c>
       <c r="C35" s="4" t="str">
         <f>'PR7_Co(OH)2_Europe_Recycling'!C118</f>
-        <v>Europe</v>
+        <v>Europe witout Switzerland</v>
       </c>
       <c r="D35" s="4">
         <v>6.2643907715534755E-3</v>
@@ -4326,7 +4318,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
@@ -4334,7 +4326,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
@@ -4342,7 +4334,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
@@ -4366,7 +4358,7 @@
         <v>7</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
@@ -4448,10 +4440,10 @@
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="B10" s="4" t="s">
         <v>143</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>144</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>25</v>
@@ -4469,7 +4461,7 @@
         <v>21</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
@@ -4495,15 +4487,15 @@
         <v>21</v>
       </c>
       <c r="J11" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="B12" s="4" t="s">
         <v>147</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>148</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>28</v>
@@ -4521,7 +4513,7 @@
         <v>21</v>
       </c>
       <c r="J12" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
@@ -4547,15 +4539,15 @@
         <v>21</v>
       </c>
       <c r="J13" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="B14" s="4" t="s">
         <v>149</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>150</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>25</v>
@@ -4573,7 +4565,7 @@
         <v>21</v>
       </c>
       <c r="J14" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
@@ -4599,7 +4591,7 @@
         <v>21</v>
       </c>
       <c r="J15" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
@@ -4625,15 +4617,15 @@
         <v>21</v>
       </c>
       <c r="J16" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="B17" s="4" t="s">
         <v>152</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>153</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>25</v>
@@ -4651,15 +4643,15 @@
         <v>21</v>
       </c>
       <c r="J17" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="B18" s="4" t="s">
         <v>154</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>155</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>25</v>
@@ -4677,7 +4669,7 @@
         <v>21</v>
       </c>
       <c r="J18" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
@@ -4688,7 +4680,7 @@
         <v>27</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D19" s="4">
         <v>11.5245</v>
@@ -4703,15 +4695,15 @@
         <v>21</v>
       </c>
       <c r="J19" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="B20" s="4" t="s">
         <v>156</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>157</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>25</v>
@@ -4729,15 +4721,15 @@
         <v>21</v>
       </c>
       <c r="J20" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="B21" s="4" t="s">
         <v>158</v>
-      </c>
-      <c r="B21" s="4" t="s">
-        <v>159</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>25</v>
@@ -4755,15 +4747,15 @@
         <v>21</v>
       </c>
       <c r="J21" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="B22" s="4" t="s">
         <v>160</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>161</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>28</v>
@@ -4781,7 +4773,7 @@
         <v>21</v>
       </c>
       <c r="J22" s="4" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
@@ -4807,15 +4799,15 @@
         <v>21</v>
       </c>
       <c r="J23" s="4" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="B24" s="4" t="s">
         <v>160</v>
-      </c>
-      <c r="B24" s="4" t="s">
-        <v>161</v>
       </c>
       <c r="C24" s="4" t="s">
         <v>28</v>
@@ -4833,15 +4825,15 @@
         <v>21</v>
       </c>
       <c r="J24" s="4" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="B25" s="4" t="s">
         <v>163</v>
-      </c>
-      <c r="B25" s="4" t="s">
-        <v>164</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>28</v>
@@ -4859,15 +4851,15 @@
         <v>21</v>
       </c>
       <c r="J25" s="4" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="B26" s="4" t="s">
         <v>165</v>
-      </c>
-      <c r="B26" s="4" t="s">
-        <v>166</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>25</v>
@@ -4885,15 +4877,15 @@
         <v>21</v>
       </c>
       <c r="J26" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="B27" s="4" t="s">
         <v>167</v>
-      </c>
-      <c r="B27" s="4" t="s">
-        <v>168</v>
       </c>
       <c r="C27" s="4" t="s">
         <v>28</v>
@@ -4911,7 +4903,7 @@
         <v>21</v>
       </c>
       <c r="J27" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
@@ -4937,15 +4929,15 @@
         <v>21</v>
       </c>
       <c r="J28" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="B29" s="4" t="s">
         <v>169</v>
-      </c>
-      <c r="B29" s="4" t="s">
-        <v>170</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>28</v>
@@ -4963,15 +4955,15 @@
         <v>21</v>
       </c>
       <c r="J29" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="B30" s="4" t="s">
         <v>171</v>
-      </c>
-      <c r="B30" s="4" t="s">
-        <v>172</v>
       </c>
       <c r="C30" s="4" t="s">
         <v>28</v>
@@ -4989,15 +4981,15 @@
         <v>21</v>
       </c>
       <c r="J30" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="B31" s="4" t="s">
         <v>173</v>
-      </c>
-      <c r="B31" s="4" t="s">
-        <v>174</v>
       </c>
       <c r="C31" s="4" t="s">
         <v>28</v>
@@ -5015,15 +5007,15 @@
         <v>21</v>
       </c>
       <c r="J31" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="B32" s="4" t="s">
         <v>175</v>
-      </c>
-      <c r="B32" s="4" t="s">
-        <v>176</v>
       </c>
       <c r="C32" s="4" t="s">
         <v>25</v>
@@ -5041,15 +5033,15 @@
         <v>21</v>
       </c>
       <c r="J32" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="B33" s="4" t="s">
         <v>177</v>
-      </c>
-      <c r="B33" s="4" t="s">
-        <v>178</v>
       </c>
       <c r="C33" s="4" t="s">
         <v>28</v>
@@ -5067,15 +5059,15 @@
         <v>21</v>
       </c>
       <c r="J33" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="B34" s="4" t="s">
         <v>179</v>
-      </c>
-      <c r="B34" s="4" t="s">
-        <v>180</v>
       </c>
       <c r="C34" s="4" t="s">
         <v>28</v>
@@ -5093,7 +5085,7 @@
         <v>21</v>
       </c>
       <c r="J34" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
@@ -5119,7 +5111,7 @@
         <v>21</v>
       </c>
       <c r="J35" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
@@ -5145,7 +5137,7 @@
         <v>21</v>
       </c>
       <c r="J36" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
@@ -5171,7 +5163,7 @@
         <v>21</v>
       </c>
       <c r="J37" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
@@ -5197,15 +5189,15 @@
         <v>21</v>
       </c>
       <c r="J38" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="B39" s="4" t="s">
         <v>181</v>
-      </c>
-      <c r="B39" s="4" t="s">
-        <v>182</v>
       </c>
       <c r="C39" s="4" t="s">
         <v>25</v>
@@ -5223,15 +5215,15 @@
         <v>21</v>
       </c>
       <c r="J39" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="B40" s="4" t="s">
         <v>184</v>
-      </c>
-      <c r="B40" s="4" t="s">
-        <v>185</v>
       </c>
       <c r="C40" s="4" t="s">
         <v>25</v>
@@ -5249,18 +5241,18 @@
         <v>21</v>
       </c>
       <c r="J40" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" s="4" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D41" s="4">
         <v>2.223E-2</v>
       </c>
       <c r="E41" s="4" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F41" s="4" t="s">
         <v>45</v>
@@ -5269,10 +5261,10 @@
         <v>46</v>
       </c>
       <c r="H41" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="J41" s="4" t="s">
         <v>188</v>
-      </c>
-      <c r="J41" s="4" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
@@ -5295,7 +5287,7 @@
         <v>47</v>
       </c>
       <c r="J42" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
@@ -5318,12 +5310,12 @@
         <v>47</v>
       </c>
       <c r="J43" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D44" s="4">
         <v>4.2009999999999999E-5</v>
@@ -5338,15 +5330,15 @@
         <v>46</v>
       </c>
       <c r="H44" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="J44" s="4" t="s">
         <v>192</v>
-      </c>
-      <c r="J44" s="4" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" s="4" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D45" s="4">
         <v>7.3300000000000006E-5</v>
@@ -5361,15 +5353,15 @@
         <v>46</v>
       </c>
       <c r="H45" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="J45" s="4" t="s">
         <v>192</v>
-      </c>
-      <c r="J45" s="4" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D46" s="4">
         <v>4.1300000000000003E-6</v>
@@ -5384,15 +5376,15 @@
         <v>46</v>
       </c>
       <c r="H46" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="J46" s="4" t="s">
         <v>192</v>
-      </c>
-      <c r="J46" s="4" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" s="4" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D47" s="4">
         <v>1.33E-6</v>
@@ -5407,15 +5399,15 @@
         <v>46</v>
       </c>
       <c r="H47" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="J47" s="4" t="s">
         <v>192</v>
-      </c>
-      <c r="J47" s="4" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="D48" s="4">
         <v>9.5799999999999998E-6</v>
@@ -5430,15 +5422,15 @@
         <v>46</v>
       </c>
       <c r="H48" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="J48" s="4" t="s">
         <v>192</v>
-      </c>
-      <c r="J48" s="4" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" s="4" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D49" s="4">
         <v>2.8999999999999998E-7</v>
@@ -5453,15 +5445,15 @@
         <v>46</v>
       </c>
       <c r="H49" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="J49" s="4" t="s">
         <v>192</v>
-      </c>
-      <c r="J49" s="4" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D50" s="4">
         <v>3.8000000000000001E-7</v>
@@ -5476,15 +5468,15 @@
         <v>46</v>
       </c>
       <c r="H50" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="J50" s="4" t="s">
         <v>192</v>
-      </c>
-      <c r="J50" s="4" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" s="4" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="D51" s="4">
         <v>7.0000000000000005E-8</v>
@@ -5499,15 +5491,15 @@
         <v>46</v>
       </c>
       <c r="H51" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="J51" s="4" t="s">
         <v>192</v>
-      </c>
-      <c r="J51" s="4" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" s="4" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D52" s="4">
         <v>4.5199999999999999E-6</v>
@@ -5522,15 +5514,15 @@
         <v>46</v>
       </c>
       <c r="H52" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="J52" s="4" t="s">
         <v>192</v>
-      </c>
-      <c r="J52" s="4" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" s="4" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D53" s="4">
         <v>5.9999999999999995E-8</v>
@@ -5545,15 +5537,15 @@
         <v>46</v>
       </c>
       <c r="H53" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="J53" s="4" t="s">
         <v>192</v>
-      </c>
-      <c r="J53" s="4" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D54" s="4">
         <v>1E-8</v>
@@ -5568,10 +5560,10 @@
         <v>46</v>
       </c>
       <c r="H54" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="J54" s="4" t="s">
         <v>192</v>
-      </c>
-      <c r="J54" s="4" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.25">
@@ -5594,12 +5586,12 @@
         <v>76</v>
       </c>
       <c r="J55" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D56" s="4">
         <v>6.6E-4</v>
@@ -5617,12 +5609,12 @@
         <v>76</v>
       </c>
       <c r="J56" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" s="4" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D57" s="4">
         <v>4.8999999999999997E-7</v>
@@ -5640,12 +5632,12 @@
         <v>76</v>
       </c>
       <c r="J57" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D58" s="4">
         <v>3.9390000000000001E-5</v>
@@ -5663,12 +5655,12 @@
         <v>76</v>
       </c>
       <c r="J58" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59" s="4" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D59" s="4">
         <v>1.6700000000000001E-6</v>
@@ -5686,12 +5678,12 @@
         <v>76</v>
       </c>
       <c r="J59" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="D60" s="4">
         <v>5.4199999999999999E-9</v>
@@ -5709,12 +5701,12 @@
         <v>76</v>
       </c>
       <c r="J60" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A61" s="4" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D61" s="4">
         <v>2.7199999999999998E-6</v>
@@ -5732,12 +5724,12 @@
         <v>76</v>
       </c>
       <c r="J61" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="D62" s="4">
         <v>1.0883999999999999E-4</v>
@@ -5752,15 +5744,15 @@
         <v>46</v>
       </c>
       <c r="H62" s="4" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="J62" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A63" s="4" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D63" s="4">
         <v>4.1670999999999999E-4</v>
@@ -5775,15 +5767,15 @@
         <v>46</v>
       </c>
       <c r="H63" s="4" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="J63" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A64" s="4" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D64" s="4">
         <v>2.7990000000000001E-5</v>
@@ -5798,15 +5790,15 @@
         <v>46</v>
       </c>
       <c r="H64" s="4" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="J64" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A65" s="4" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D65" s="4">
         <v>4.6650000000000002E-5</v>
@@ -5821,15 +5813,15 @@
         <v>46</v>
       </c>
       <c r="H65" s="4" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="J65" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A66" s="4" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D66" s="4">
         <v>1.0883999999999999E-4</v>
@@ -5844,10 +5836,10 @@
         <v>46</v>
       </c>
       <c r="H66" s="4" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="J66" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="67" spans="1:14" s="9" customFormat="1" x14ac:dyDescent="0.25"/>
@@ -5856,7 +5848,7 @@
         <v>0</v>
       </c>
       <c r="B68" s="13" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="69" spans="1:14" x14ac:dyDescent="0.25">
@@ -5864,7 +5856,7 @@
         <v>1</v>
       </c>
       <c r="B69" s="4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="70" spans="1:14" x14ac:dyDescent="0.25">
@@ -5872,7 +5864,7 @@
         <v>2</v>
       </c>
       <c r="B70" s="4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="71" spans="1:14" x14ac:dyDescent="0.25">
@@ -6010,7 +6002,7 @@
         <v>0</v>
       </c>
       <c r="B79" s="13" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="80" spans="1:14" x14ac:dyDescent="0.25">
@@ -6018,7 +6010,7 @@
         <v>1</v>
       </c>
       <c r="B80" s="4" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="81" spans="1:14" x14ac:dyDescent="0.25">
@@ -6026,7 +6018,7 @@
         <v>2</v>
       </c>
       <c r="B81" s="4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="82" spans="1:14" x14ac:dyDescent="0.25">
@@ -6192,7 +6184,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
@@ -6200,7 +6192,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
@@ -6208,7 +6200,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
@@ -6363,7 +6355,7 @@
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D12" s="4">
         <v>1.4400000000000001E-3</v>
@@ -6386,7 +6378,7 @@
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D13" s="4">
         <v>1.4799999999999999E-4</v>
@@ -6436,7 +6428,7 @@
         <v>0</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
@@ -6444,7 +6436,7 @@
         <v>1</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
@@ -6452,7 +6444,7 @@
         <v>2</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.25">
@@ -6476,7 +6468,7 @@
         <v>7</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.25">
@@ -6563,7 +6555,7 @@
         <v>27</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D25" s="4">
         <v>8.345257017438195</v>
@@ -6635,10 +6627,10 @@
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="B28" s="4" t="s">
         <v>122</v>
-      </c>
-      <c r="B28" s="4" t="s">
-        <v>123</v>
       </c>
       <c r="C28" s="4" t="s">
         <v>25</v>
@@ -6687,10 +6679,10 @@
     </row>
     <row r="30" spans="1:14" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="B30" s="10" t="s">
         <v>124</v>
-      </c>
-      <c r="B30" s="10" t="s">
-        <v>125</v>
       </c>
       <c r="C30" s="10" t="s">
         <v>28</v>
@@ -6736,7 +6728,7 @@
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D32" s="4">
         <v>2.7920252309287196E-2</v>
@@ -6763,7 +6755,7 @@
         <v>0</v>
       </c>
       <c r="B34" s="13" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.25">
@@ -6771,7 +6763,7 @@
         <v>1</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.25">
@@ -6779,7 +6771,7 @@
         <v>2</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.25">
@@ -6891,7 +6883,7 @@
         <v>53</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D43" s="4">
         <v>3.5072393888888893E-2</v>
@@ -6906,15 +6898,15 @@
         <v>21</v>
       </c>
       <c r="J43" s="4" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="B44" s="4" t="s">
         <v>219</v>
-      </c>
-      <c r="B44" s="4" t="s">
-        <v>220</v>
       </c>
       <c r="C44" s="4" t="s">
         <v>25</v>
@@ -6932,7 +6924,7 @@
         <v>21</v>
       </c>
       <c r="J44" s="4" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.25">
@@ -6943,7 +6935,7 @@
         <v>27</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D45" s="4">
         <v>1.269868</v>
@@ -6958,7 +6950,7 @@
         <v>21</v>
       </c>
       <c r="J45" s="4" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.25">
@@ -6984,7 +6976,7 @@
         <v>21</v>
       </c>
       <c r="J46" s="4" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.25">
@@ -7010,15 +7002,15 @@
         <v>21</v>
       </c>
       <c r="J47" s="4" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="B48" s="4" t="s">
         <v>149</v>
-      </c>
-      <c r="B48" s="4" t="s">
-        <v>150</v>
       </c>
       <c r="C48" s="4" t="s">
         <v>25</v>
@@ -7036,7 +7028,7 @@
         <v>21</v>
       </c>
       <c r="J48" s="4" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.25">
@@ -7062,15 +7054,15 @@
         <v>21</v>
       </c>
       <c r="J49" s="4" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="B50" s="4" t="s">
         <v>122</v>
-      </c>
-      <c r="B50" s="4" t="s">
-        <v>123</v>
       </c>
       <c r="C50" s="4" t="s">
         <v>25</v>
@@ -7088,15 +7080,15 @@
         <v>21</v>
       </c>
       <c r="J50" s="4" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="B51" s="4" t="s">
         <v>154</v>
-      </c>
-      <c r="B51" s="4" t="s">
-        <v>155</v>
       </c>
       <c r="C51" s="4" t="s">
         <v>25</v>
@@ -7114,7 +7106,7 @@
         <v>21</v>
       </c>
       <c r="J51" s="4" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.25">
@@ -7140,7 +7132,7 @@
         <v>21</v>
       </c>
       <c r="J52" s="4" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.25">
@@ -7166,15 +7158,15 @@
         <v>21</v>
       </c>
       <c r="J53" s="4" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="B54" s="4" t="s">
         <v>175</v>
-      </c>
-      <c r="B54" s="4" t="s">
-        <v>176</v>
       </c>
       <c r="C54" s="4" t="s">
         <v>25</v>
@@ -7192,15 +7184,15 @@
         <v>21</v>
       </c>
       <c r="J54" s="4" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="B55" s="4" t="s">
         <v>152</v>
-      </c>
-      <c r="B55" s="4" t="s">
-        <v>153</v>
       </c>
       <c r="C55" s="4" t="s">
         <v>25</v>
@@ -7218,15 +7210,15 @@
         <v>21</v>
       </c>
       <c r="J55" s="4" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="B56" s="4" t="s">
         <v>147</v>
-      </c>
-      <c r="B56" s="4" t="s">
-        <v>148</v>
       </c>
       <c r="C56" s="4" t="s">
         <v>28</v>
@@ -7244,7 +7236,7 @@
         <v>21</v>
       </c>
       <c r="J56" s="4" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.25">
@@ -7267,7 +7259,7 @@
         <v>47</v>
       </c>
       <c r="J57" s="4" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="58" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25"/>
@@ -7276,7 +7268,7 @@
         <v>0</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.25">
@@ -7284,7 +7276,7 @@
         <v>1</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.25">
@@ -7292,7 +7284,7 @@
         <v>2</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>222</v>
+        <v>141</v>
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.25">
@@ -7316,7 +7308,7 @@
         <v>7</v>
       </c>
       <c r="B64" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.25">
@@ -7377,9 +7369,8 @@
         <f>B60</f>
         <v>CoSO4</v>
       </c>
-      <c r="C67" s="4" t="str">
-        <f>B61</f>
-        <v>CD-CN</v>
+      <c r="C67" s="4" t="s">
+        <v>141</v>
       </c>
       <c r="D67" s="4">
         <v>1</v>
@@ -7486,7 +7477,7 @@
         <v>0</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
     </row>
     <row r="73" spans="1:14" x14ac:dyDescent="0.25">
@@ -7494,7 +7485,7 @@
         <v>1</v>
       </c>
       <c r="B73" s="4" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="74" spans="1:14" x14ac:dyDescent="0.25">
@@ -7502,7 +7493,7 @@
         <v>2</v>
       </c>
       <c r="B74" s="4" t="s">
-        <v>222</v>
+        <v>141</v>
       </c>
     </row>
     <row r="75" spans="1:14" x14ac:dyDescent="0.25">
@@ -7526,7 +7517,7 @@
         <v>7</v>
       </c>
       <c r="B77" s="8" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
     </row>
     <row r="78" spans="1:14" x14ac:dyDescent="0.25">
@@ -7587,9 +7578,8 @@
         <f>B73</f>
         <v>CoSO4 (Co content)</v>
       </c>
-      <c r="C80" s="4" t="str">
-        <f>B74</f>
-        <v>CD-CN</v>
+      <c r="C80" s="4" t="s">
+        <v>141</v>
       </c>
       <c r="D80" s="4">
         <v>1</v>
@@ -7724,7 +7714,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
@@ -7732,7 +7722,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
@@ -7740,7 +7730,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
@@ -7852,7 +7842,7 @@
         <v>53</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D10" s="15">
         <v>5.2442857142857152E-2</v>
@@ -7867,15 +7857,15 @@
         <v>21</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>219</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>220</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>25</v>
@@ -7893,7 +7883,7 @@
         <v>21</v>
       </c>
       <c r="J11" s="4" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
@@ -7904,7 +7894,7 @@
         <v>27</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D12" s="15">
         <v>2.517257142857143E-2</v>
@@ -7919,15 +7909,15 @@
         <v>21</v>
       </c>
       <c r="J12" s="4" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>28</v>
@@ -7945,7 +7935,7 @@
         <v>21</v>
       </c>
       <c r="J13" s="4" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
@@ -7971,15 +7961,15 @@
         <v>21</v>
       </c>
       <c r="J14" s="4" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>28</v>
@@ -7997,15 +7987,15 @@
         <v>21</v>
       </c>
       <c r="J15" s="4" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="B16" s="4" t="s">
         <v>152</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>153</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>25</v>
@@ -8023,7 +8013,7 @@
         <v>21</v>
       </c>
       <c r="J16" s="4" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
@@ -8046,7 +8036,7 @@
         <v>47</v>
       </c>
       <c r="J17" s="4" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
@@ -8069,7 +8059,7 @@
         <v>76</v>
       </c>
       <c r="J18" s="4" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="19" spans="1:14" s="9" customFormat="1" x14ac:dyDescent="0.25"/>
@@ -8078,7 +8068,7 @@
         <v>0</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.25">
@@ -8086,7 +8076,7 @@
         <v>1</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.25">
@@ -8094,7 +8084,7 @@
         <v>2</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>222</v>
+        <v>141</v>
       </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.25">
@@ -8118,7 +8108,7 @@
         <v>7</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.25">
@@ -8179,9 +8169,8 @@
         <f>B21</f>
         <v>Co3O4</v>
       </c>
-      <c r="C28" s="4" t="str">
-        <f>B22</f>
-        <v>CD-CN</v>
+      <c r="C28" s="4" t="s">
+        <v>141</v>
       </c>
       <c r="D28" s="4">
         <v>1</v>
@@ -8316,7 +8305,7 @@
         <v>0</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.25">
@@ -8324,7 +8313,7 @@
         <v>1</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.25">
@@ -8332,7 +8321,7 @@
         <v>2</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>222</v>
+        <v>141</v>
       </c>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.25">
@@ -8356,7 +8345,7 @@
         <v>7</v>
       </c>
       <c r="B39" s="14" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.25">
@@ -8417,9 +8406,8 @@
         <f>B35</f>
         <v>Co3O4 (Co content)</v>
       </c>
-      <c r="C42" s="4" t="str">
-        <f>B36</f>
-        <v>CD-CN</v>
+      <c r="C42" s="4" t="s">
+        <v>141</v>
       </c>
       <c r="D42" s="4">
         <v>1</v>
@@ -8589,7 +8577,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
@@ -8597,7 +8585,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
@@ -8717,7 +8705,7 @@
         <v>27</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D10" s="4">
         <v>3.4</v>
@@ -8732,7 +8720,7 @@
         <v>21</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
     </row>
     <row r="11" spans="1:14" s="9" customFormat="1" x14ac:dyDescent="0.25"/>
@@ -8741,7 +8729,7 @@
         <v>0</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
@@ -8749,7 +8737,7 @@
         <v>1</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
@@ -8757,7 +8745,7 @@
         <v>2</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>241</v>
+        <v>141</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
@@ -8781,7 +8769,7 @@
         <v>7</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
@@ -8842,9 +8830,8 @@
         <f>B13</f>
         <v>Co metal</v>
       </c>
-      <c r="C20" s="4" t="str">
-        <f>B14</f>
-        <v>CD-CN-GLO</v>
+      <c r="C20" s="4" t="s">
+        <v>141</v>
       </c>
       <c r="D20" s="4">
         <v>1</v>
@@ -9047,7 +9034,7 @@
         <v>7</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
@@ -9587,7 +9574,7 @@
         <v>7</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
@@ -9840,7 +9827,7 @@
         <v>7</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.25">
@@ -10355,7 +10342,7 @@
         <v>7</v>
       </c>
       <c r="B46" s="8" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.25">
@@ -10542,7 +10529,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>97</v>
+        <v>253</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
@@ -10629,7 +10616,7 @@
       </c>
       <c r="C9" s="4" t="str">
         <f>B3</f>
-        <v>Europe</v>
+        <v>Europe witout Switzerland</v>
       </c>
       <c r="D9" s="4">
         <v>1</v>
@@ -10654,7 +10641,7 @@
         <v>59</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D10" s="4">
         <v>0.25315091723266886</v>
@@ -10669,7 +10656,7 @@
         <v>21</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
@@ -10680,7 +10667,7 @@
         <v>81</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D11" s="4">
         <v>15.29988253062595</v>
@@ -10695,7 +10682,7 @@
         <v>21</v>
       </c>
       <c r="J11" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
@@ -10706,7 +10693,7 @@
         <v>27</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D12" s="4">
         <v>0.30700552240308782</v>
@@ -10721,12 +10708,12 @@
         <v>21</v>
       </c>
       <c r="J12" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D13" s="4">
         <v>0.1683168316831683</v>
@@ -10744,7 +10731,7 @@
         <v>76</v>
       </c>
       <c r="J13" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
@@ -10767,7 +10754,7 @@
         <v>76</v>
       </c>
       <c r="J14" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
@@ -10790,7 +10777,7 @@
         <v>76</v>
       </c>
       <c r="J15" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="16" spans="1:14" s="11" customFormat="1" x14ac:dyDescent="0.25"/>
@@ -10799,7 +10786,7 @@
         <v>0</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
@@ -10807,7 +10794,7 @@
         <v>1</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.25">
@@ -10815,7 +10802,7 @@
         <v>2</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>97</v>
+        <v>253</v>
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.25">
@@ -10839,7 +10826,7 @@
         <v>7</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.25">
@@ -10902,7 +10889,7 @@
       </c>
       <c r="C25" s="4" t="str">
         <f>B19</f>
-        <v>Europe</v>
+        <v>Europe witout Switzerland</v>
       </c>
       <c r="D25" s="4">
         <v>1</v>
@@ -10927,7 +10914,7 @@
         <v>75</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D26" s="8">
         <v>0.23320908059371151</v>
@@ -10942,7 +10929,7 @@
         <v>21</v>
       </c>
       <c r="J26" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.25">
@@ -10953,7 +10940,7 @@
         <v>69</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D27" s="8">
         <v>0.10542328300811614</v>
@@ -10968,7 +10955,7 @@
         <v>21</v>
       </c>
       <c r="J27" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.25">
@@ -10979,7 +10966,7 @@
         <v>27</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D28" s="8">
         <v>5.6255913807107767E-2</v>
@@ -10994,7 +10981,7 @@
         <v>21</v>
       </c>
       <c r="J28" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.25">
@@ -11017,7 +11004,7 @@
         <v>76</v>
       </c>
       <c r="J29" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="30" spans="1:14" s="11" customFormat="1" x14ac:dyDescent="0.25"/>
@@ -11026,7 +11013,7 @@
         <v>0</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.25">
@@ -11034,7 +11021,7 @@
         <v>1</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.25">
@@ -11042,7 +11029,7 @@
         <v>2</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>97</v>
+        <v>253</v>
       </c>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.25">
@@ -11129,7 +11116,7 @@
       </c>
       <c r="C39" s="4" t="str">
         <f>B33</f>
-        <v>Europe</v>
+        <v>Europe witout Switzerland</v>
       </c>
       <c r="D39" s="4">
         <v>1</v>
@@ -11154,7 +11141,7 @@
         <v>75</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D40" s="4">
         <v>0.7953277285916226</v>
@@ -11169,7 +11156,7 @@
         <v>21</v>
       </c>
       <c r="J40" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.25">
@@ -11180,7 +11167,7 @@
         <v>67</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D41" s="4">
         <v>0.19986112144433699</v>
@@ -11195,7 +11182,7 @@
         <v>21</v>
       </c>
       <c r="J41" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.25">
@@ -11206,7 +11193,7 @@
         <v>83</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D42" s="4">
         <v>1.034149244847854E-2</v>
@@ -11221,7 +11208,7 @@
         <v>21</v>
       </c>
       <c r="J42" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.25">
@@ -11232,7 +11219,7 @@
         <v>27</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D43" s="4">
         <v>1.3426315551918261E-2</v>
@@ -11247,15 +11234,15 @@
         <v>21</v>
       </c>
       <c r="J43" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="B44" s="4" t="s">
         <v>102</v>
-      </c>
-      <c r="B44" s="4" t="s">
-        <v>103</v>
       </c>
       <c r="C44" s="4" t="s">
         <v>25</v>
@@ -11273,7 +11260,7 @@
         <v>21</v>
       </c>
       <c r="J44" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.25">
@@ -11296,7 +11283,7 @@
         <v>76</v>
       </c>
       <c r="J45" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="46" spans="1:14" s="11" customFormat="1" x14ac:dyDescent="0.25"/>
@@ -11305,7 +11292,7 @@
         <v>0</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.25">
@@ -11313,7 +11300,7 @@
         <v>1</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.25">
@@ -11321,7 +11308,7 @@
         <v>2</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>97</v>
+        <v>253</v>
       </c>
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.25">
@@ -11408,7 +11395,7 @@
       </c>
       <c r="C55" s="4" t="str">
         <f>B49</f>
-        <v>Europe</v>
+        <v>Europe witout Switzerland</v>
       </c>
       <c r="D55" s="4">
         <v>1</v>
@@ -11433,7 +11420,7 @@
         <v>75</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D56" s="4">
         <v>0.36423560630654789</v>
@@ -11448,7 +11435,7 @@
         <v>21</v>
       </c>
       <c r="J56" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.25">
@@ -11459,7 +11446,7 @@
         <v>69</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D57" s="4">
         <v>7.1125100568831423E-2</v>
@@ -11474,7 +11461,7 @@
         <v>21</v>
       </c>
       <c r="J57" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="58" spans="1:14" x14ac:dyDescent="0.25">
@@ -11485,7 +11472,7 @@
         <v>27</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D58" s="4">
         <v>4.8688684122122322E-2</v>
@@ -11500,15 +11487,15 @@
         <v>21</v>
       </c>
       <c r="J58" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A59" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="B59" s="4" t="s">
         <v>102</v>
-      </c>
-      <c r="B59" s="4" t="s">
-        <v>103</v>
       </c>
       <c r="C59" s="4" t="s">
         <v>25</v>
@@ -11526,7 +11513,7 @@
         <v>21</v>
       </c>
       <c r="J59" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="60" spans="1:14" x14ac:dyDescent="0.25">
@@ -11549,7 +11536,7 @@
         <v>76</v>
       </c>
       <c r="J60" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="61" spans="1:14" s="11" customFormat="1" x14ac:dyDescent="0.25"/>
@@ -11558,7 +11545,7 @@
         <v>0</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="63" spans="1:14" x14ac:dyDescent="0.25">
@@ -11566,7 +11553,7 @@
         <v>1</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.25">
@@ -11574,7 +11561,7 @@
         <v>2</v>
       </c>
       <c r="B64" s="4" t="s">
-        <v>97</v>
+        <v>253</v>
       </c>
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.25">
@@ -11661,7 +11648,7 @@
       </c>
       <c r="C70" s="4" t="str">
         <f>B64</f>
-        <v>Europe</v>
+        <v>Europe witout Switzerland</v>
       </c>
       <c r="D70" s="4">
         <v>1</v>
@@ -11686,7 +11673,7 @@
         <v>75</v>
       </c>
       <c r="C71" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D71" s="4">
         <v>6.0030413625304133</v>
@@ -11701,7 +11688,7 @@
         <v>21</v>
       </c>
       <c r="J71" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="72" spans="1:14" x14ac:dyDescent="0.25">
@@ -11712,7 +11699,7 @@
         <v>69</v>
       </c>
       <c r="C72" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D72" s="4">
         <v>0.86374695863746953</v>
@@ -11727,7 +11714,7 @@
         <v>21</v>
       </c>
       <c r="J72" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="73" spans="1:14" x14ac:dyDescent="0.25">
@@ -11738,7 +11725,7 @@
         <v>27</v>
       </c>
       <c r="C73" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D73" s="4">
         <v>3.4554974927007298</v>
@@ -11753,7 +11740,7 @@
         <v>21</v>
       </c>
       <c r="J73" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="74" spans="1:14" x14ac:dyDescent="0.25">
@@ -11762,12 +11749,11 @@
         <v>Effluent treatment</v>
       </c>
       <c r="B74" s="4" t="str">
-        <f t="shared" ref="B74:C74" si="0">B85</f>
+        <f t="shared" ref="B74" si="0">B85</f>
         <v>Wastewater</v>
       </c>
-      <c r="C74" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>Europe</v>
+      <c r="C74" s="4" t="s">
+        <v>253</v>
       </c>
       <c r="D74" s="4">
         <v>49.996958637469596</v>
@@ -11784,7 +11770,7 @@
         <v>21</v>
       </c>
       <c r="J74" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="75" spans="1:14" x14ac:dyDescent="0.25">
@@ -11807,7 +11793,7 @@
         <v>76</v>
       </c>
       <c r="J75" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="76" spans="1:14" s="11" customFormat="1" x14ac:dyDescent="0.25"/>
@@ -11816,7 +11802,7 @@
         <v>0</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="78" spans="1:14" x14ac:dyDescent="0.25">
@@ -11824,7 +11810,7 @@
         <v>1</v>
       </c>
       <c r="B78" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="79" spans="1:14" x14ac:dyDescent="0.25">
@@ -11832,7 +11818,7 @@
         <v>2</v>
       </c>
       <c r="B79" s="4" t="s">
-        <v>97</v>
+        <v>253</v>
       </c>
     </row>
     <row r="80" spans="1:14" x14ac:dyDescent="0.25">
@@ -11919,7 +11905,7 @@
       </c>
       <c r="C85" s="4" t="str">
         <f>B79</f>
-        <v>Europe</v>
+        <v>Europe witout Switzerland</v>
       </c>
       <c r="D85" s="4">
         <v>1</v>
@@ -11959,18 +11945,18 @@
         <v>21</v>
       </c>
       <c r="J86" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="87" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A87" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="B87" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="B87" s="4" t="s">
-        <v>107</v>
-      </c>
       <c r="C87" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D87" s="4">
         <v>7.8877827641980099E-3</v>
@@ -11985,7 +11971,7 @@
         <v>21</v>
       </c>
       <c r="J87" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="88" spans="1:14" x14ac:dyDescent="0.25">
@@ -11996,7 +11982,7 @@
         <v>67</v>
       </c>
       <c r="C88" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D88" s="4">
         <v>2.8082784700549011E-2</v>
@@ -12011,7 +11997,7 @@
         <v>21</v>
       </c>
       <c r="J88" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="89" spans="1:14" x14ac:dyDescent="0.25">
@@ -12022,7 +12008,7 @@
         <v>75</v>
       </c>
       <c r="C89" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D89" s="4">
         <v>0.18377110053078799</v>
@@ -12037,7 +12023,7 @@
         <v>21</v>
       </c>
       <c r="J89" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="90" spans="1:14" x14ac:dyDescent="0.25">
@@ -12048,7 +12034,7 @@
         <v>27</v>
       </c>
       <c r="C90" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D90" s="4">
         <v>4.1791360605508351E-2</v>
@@ -12063,7 +12049,7 @@
         <v>21</v>
       </c>
       <c r="J90" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="91" spans="1:14" x14ac:dyDescent="0.25">
@@ -12074,7 +12060,7 @@
         <v>73</v>
       </c>
       <c r="C91" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D91" s="4">
         <v>-9.6548169578786712E-4</v>
@@ -12089,15 +12075,15 @@
         <v>21</v>
       </c>
       <c r="J91" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="92" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A92" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="B92" s="4" t="s">
         <v>102</v>
-      </c>
-      <c r="B92" s="4" t="s">
-        <v>103</v>
       </c>
       <c r="C92" s="4" t="s">
         <v>25</v>
@@ -12115,7 +12101,7 @@
         <v>21</v>
       </c>
       <c r="J92" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="93" spans="1:14" x14ac:dyDescent="0.25">
@@ -12138,7 +12124,7 @@
         <v>76</v>
       </c>
       <c r="J93" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="94" spans="1:14" s="9" customFormat="1" x14ac:dyDescent="0.25"/>
@@ -12147,7 +12133,7 @@
         <v>0</v>
       </c>
       <c r="B95" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="96" spans="1:14" x14ac:dyDescent="0.25">
@@ -12155,7 +12141,7 @@
         <v>1</v>
       </c>
       <c r="B96" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="97" spans="1:14" x14ac:dyDescent="0.25">
@@ -12163,7 +12149,7 @@
         <v>2</v>
       </c>
       <c r="B97" s="4" t="s">
-        <v>97</v>
+        <v>253</v>
       </c>
     </row>
     <row r="98" spans="1:14" x14ac:dyDescent="0.25">
@@ -12187,7 +12173,7 @@
         <v>7</v>
       </c>
       <c r="B100" s="8" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="101" spans="1:14" x14ac:dyDescent="0.25">
@@ -12250,7 +12236,7 @@
       </c>
       <c r="C103" s="4" t="str">
         <f>B97</f>
-        <v>Europe</v>
+        <v>Europe witout Switzerland</v>
       </c>
       <c r="D103" s="4">
         <v>1</v>
@@ -12276,7 +12262,7 @@
       </c>
       <c r="C104" s="4" t="str">
         <f t="shared" si="2"/>
-        <v>Europe</v>
+        <v>Europe witout Switzerland</v>
       </c>
       <c r="D104" s="4">
         <v>1</v>
@@ -12304,7 +12290,7 @@
       </c>
       <c r="C105" s="4" t="str">
         <f t="shared" si="4"/>
-        <v>Europe</v>
+        <v>Europe witout Switzerland</v>
       </c>
       <c r="D105" s="4">
         <v>43.094282238442823</v>
@@ -12332,7 +12318,7 @@
       </c>
       <c r="C106" s="4" t="str">
         <f t="shared" si="6"/>
-        <v>Europe</v>
+        <v>Europe witout Switzerland</v>
       </c>
       <c r="D106" s="4">
         <v>24.527372262773724</v>
@@ -12360,7 +12346,7 @@
       </c>
       <c r="C107" s="4" t="str">
         <f t="shared" si="8"/>
-        <v>Europe</v>
+        <v>Europe witout Switzerland</v>
       </c>
       <c r="D107" s="4">
         <v>2.7074209245742091</v>
@@ -12388,7 +12374,7 @@
       </c>
       <c r="C108" s="4" t="str">
         <f t="shared" si="10"/>
-        <v>Europe</v>
+        <v>Europe witout Switzerland</v>
       </c>
       <c r="D108" s="8">
         <v>1.0412297403271511</v>
@@ -12411,7 +12397,7 @@
         <v>0</v>
       </c>
       <c r="B110" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="111" spans="1:14" x14ac:dyDescent="0.25">
@@ -12419,7 +12405,7 @@
         <v>1</v>
       </c>
       <c r="B111" s="4" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="112" spans="1:14" x14ac:dyDescent="0.25">
@@ -12427,7 +12413,7 @@
         <v>2</v>
       </c>
       <c r="B112" s="4" t="s">
-        <v>97</v>
+        <v>253</v>
       </c>
     </row>
     <row r="113" spans="1:14" x14ac:dyDescent="0.25">
@@ -12451,7 +12437,7 @@
         <v>7</v>
       </c>
       <c r="B115" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="116" spans="1:14" x14ac:dyDescent="0.25">
@@ -12514,7 +12500,7 @@
       </c>
       <c r="C118" s="4" t="str">
         <f>B112</f>
-        <v>Europe</v>
+        <v>Europe witout Switzerland</v>
       </c>
       <c r="D118" s="4">
         <v>1</v>
@@ -12540,7 +12526,7 @@
       </c>
       <c r="C119" s="4" t="str">
         <f t="shared" si="12"/>
-        <v>Europe</v>
+        <v>Europe witout Switzerland</v>
       </c>
       <c r="D119" s="4">
         <v>1.5772870662460567</v>
@@ -12568,7 +12554,7 @@
       </c>
       <c r="C120" s="4" t="str">
         <f t="shared" si="14"/>
-        <v>Europe</v>
+        <v>Europe witout Switzerland</v>
       </c>
       <c r="D120" s="4">
         <v>67.972054003853032</v>
@@ -12596,7 +12582,7 @@
       </c>
       <c r="C121" s="4" t="str">
         <f t="shared" si="16"/>
-        <v>Europe</v>
+        <v>Europe witout Switzerland</v>
       </c>
       <c r="D121" s="4">
         <v>38.686707039075273</v>
@@ -12624,7 +12610,7 @@
       </c>
       <c r="C122" s="4" t="str">
         <f t="shared" si="18"/>
-        <v>Europe</v>
+        <v>Europe witout Switzerland</v>
       </c>
       <c r="D122" s="4">
         <v>4.2703800072148406</v>
@@ -12652,7 +12638,7 @@
       </c>
       <c r="C123" s="4" t="str">
         <f t="shared" si="20"/>
-        <v>Europe</v>
+        <v>Europe witout Switzerland</v>
       </c>
       <c r="D123" s="8">
         <v>1.6423182024087557</v>

</xml_diff>